<commit_message>
Add Lesson 4 practice data and A4 vocabulary cards
</commit_message>
<xml_diff>
--- a/data/Lesson_1-3_英文單字_繁中注音_總表.xlsx
+++ b/data/Lesson_1-3_英文單字_繁中注音_總表.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall" sheetId="1" r:id="Rd5121f8b34604f2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 1" sheetId="2" r:id="R7c287aa254954458"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 2" sheetId="3" r:id="R653b666b021b4956"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 3" sheetId="4" r:id="R0c90974510924170"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall" sheetId="1" r:id="R5d8db633a06844e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 1" sheetId="2" r:id="Rfdd9ef3223d94b2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 2" sheetId="3" r:id="R4796b8275fe4478e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 3" sheetId="4" r:id="Rc6188ba6978c43eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 4" sheetId="5" r:id="R3e52a9bffa4e4d4c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -148,7 +149,25 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="7">
+  <x:dxfs count="9">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C6500"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF3F8FC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -219,7 +238,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OverallTable" displayName="OverallTable" ref="A4:F191" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OverallTable" displayName="OverallTable" ref="A4:F249" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="課程"/>
     <x:tableColumn id="2" name="編號"/>
@@ -260,6 +279,19 @@
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Lesson3Table" displayName="Lesson3Table" ref="A4:E42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="編號"/>
+    <x:tableColumn id="2" name="英文"/>
+    <x:tableColumn id="3" name="繁體中文"/>
+    <x:tableColumn id="4" name="注音"/>
+    <x:tableColumn id="5" name="重複標記"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Lesson4Table" displayName="Lesson4Table" ref="A4:E62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="編號"/>
     <x:tableColumn id="2" name="英文"/>
@@ -479,7 +511,7 @@
   <x:sheetData>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>Lesson 1～3 英文單字 Overall 總表</x:v>
+        <x:v>Lesson 1～4 英文單字 Overall 總表</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3920,18 +3952,1074 @@
         <x:v>ㄌㄧㄢˋ ㄒㄧˊ</x:v>
       </x:c>
       <x:c r="F191" s="15" t="str"/>
+    </x:row>
+    <x:row r="192" ht="15" hidden="0" customHeight="1">
+      <x:c r="A192" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B192" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C192" s="16" t="str">
+        <x:v>take a look</x:v>
+      </x:c>
+      <x:c r="D192" s="16" t="str">
+        <x:v>看一看</x:v>
+      </x:c>
+      <x:c r="E192" s="16" t="str">
+        <x:v>ㄎㄢˋ ㄧˊ ㄎㄢˋ</x:v>
+      </x:c>
+      <x:c r="F192" s="15" t="str"/>
+    </x:row>
+    <x:row r="193" ht="15" hidden="0" customHeight="1">
+      <x:c r="A193" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B193" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C193" s="16" t="str">
+        <x:v>shirt</x:v>
+      </x:c>
+      <x:c r="D193" s="16" t="str">
+        <x:v>襯衫</x:v>
+      </x:c>
+      <x:c r="E193" s="16" t="str">
+        <x:v>ㄔㄣˋ ㄕㄢ</x:v>
+      </x:c>
+      <x:c r="F193" s="15" t="str"/>
+    </x:row>
+    <x:row r="194" ht="15" hidden="0" customHeight="1">
+      <x:c r="A194" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B194" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C194" s="16" t="str">
+        <x:v>shelf</x:v>
+      </x:c>
+      <x:c r="D194" s="16" t="str">
+        <x:v>架子</x:v>
+      </x:c>
+      <x:c r="E194" s="16" t="str">
+        <x:v>ㄐㄧㄚˋ ㄗ˙</x:v>
+      </x:c>
+      <x:c r="F194" s="15" t="str"/>
+    </x:row>
+    <x:row r="195" ht="15" hidden="0" customHeight="1">
+      <x:c r="A195" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B195" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C195" s="16" t="str">
+        <x:v>flower</x:v>
+      </x:c>
+      <x:c r="D195" s="16" t="str">
+        <x:v>花</x:v>
+      </x:c>
+      <x:c r="E195" s="16" t="str">
+        <x:v>ㄏㄨㄚ</x:v>
+      </x:c>
+      <x:c r="F195" s="15" t="str"/>
+    </x:row>
+    <x:row r="196" ht="15" hidden="0" customHeight="1">
+      <x:c r="A196" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B196" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C196" s="16" t="str">
+        <x:v>wear / wearing</x:v>
+      </x:c>
+      <x:c r="D196" s="16" t="str">
+        <x:v>穿／正在穿</x:v>
+      </x:c>
+      <x:c r="E196" s="16" t="str">
+        <x:v>ㄔㄨㄢ／ㄓㄥˋ ㄗㄞˋ ㄔㄨㄢ</x:v>
+      </x:c>
+      <x:c r="F196" s="15" t="str"/>
+    </x:row>
+    <x:row r="197" ht="15" hidden="0" customHeight="1">
+      <x:c r="A197" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B197" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C197" s="16" t="str">
+        <x:v>jacket</x:v>
+      </x:c>
+      <x:c r="D197" s="16" t="str">
+        <x:v>夾克、外套</x:v>
+      </x:c>
+      <x:c r="E197" s="16" t="str">
+        <x:v>ㄐㄧㄚˊ ㄎㄜˋ、ㄨㄞˋ ㄊㄠˋ</x:v>
+      </x:c>
+      <x:c r="F197" s="15" t="str"/>
+    </x:row>
+    <x:row r="198" ht="15" hidden="0" customHeight="1">
+      <x:c r="A198" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B198" s="15" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C198" s="16" t="str">
+        <x:v>red</x:v>
+      </x:c>
+      <x:c r="D198" s="16" t="str">
+        <x:v>紅色</x:v>
+      </x:c>
+      <x:c r="E198" s="16" t="str">
+        <x:v>ㄏㄨㄥˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="F198" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="15" hidden="0" customHeight="1">
+      <x:c r="A199" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B199" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C199" s="16" t="str">
+        <x:v>yellow</x:v>
+      </x:c>
+      <x:c r="D199" s="16" t="str">
+        <x:v>黃色</x:v>
+      </x:c>
+      <x:c r="E199" s="16" t="str">
+        <x:v>ㄏㄨㄤˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="F199" s="15" t="str"/>
+    </x:row>
+    <x:row r="200" ht="15" hidden="0" customHeight="1">
+      <x:c r="A200" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B200" s="15" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C200" s="16" t="str">
+        <x:v>blue</x:v>
+      </x:c>
+      <x:c r="D200" s="16" t="str">
+        <x:v>藍色</x:v>
+      </x:c>
+      <x:c r="E200" s="16" t="str">
+        <x:v>ㄌㄢˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="F200" s="15" t="str"/>
+    </x:row>
+    <x:row r="201" ht="15" hidden="0" customHeight="1">
+      <x:c r="A201" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B201" s="15" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C201" s="16" t="str">
+        <x:v>green</x:v>
+      </x:c>
+      <x:c r="D201" s="16" t="str">
+        <x:v>綠色</x:v>
+      </x:c>
+      <x:c r="E201" s="16" t="str">
+        <x:v>ㄌㄩˋ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="F201" s="15" t="str"/>
+    </x:row>
+    <x:row r="202" ht="15" hidden="0" customHeight="1">
+      <x:c r="A202" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B202" s="15" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C202" s="16" t="str">
+        <x:v>orange</x:v>
+      </x:c>
+      <x:c r="D202" s="16" t="str">
+        <x:v>橘色</x:v>
+      </x:c>
+      <x:c r="E202" s="16" t="str">
+        <x:v>ㄐㄩˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="F202" s="15" t="str"/>
+    </x:row>
+    <x:row r="203" ht="15" hidden="0" customHeight="1">
+      <x:c r="A203" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B203" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C203" s="16" t="str">
+        <x:v>white</x:v>
+      </x:c>
+      <x:c r="D203" s="16" t="str">
+        <x:v>白色</x:v>
+      </x:c>
+      <x:c r="E203" s="16" t="str">
+        <x:v>ㄅㄞˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="F203" s="15" t="str"/>
+    </x:row>
+    <x:row r="204" ht="15" hidden="0" customHeight="1">
+      <x:c r="A204" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B204" s="15" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C204" s="16" t="str">
+        <x:v>black</x:v>
+      </x:c>
+      <x:c r="D204" s="16" t="str">
+        <x:v>黑色</x:v>
+      </x:c>
+      <x:c r="E204" s="16" t="str">
+        <x:v>ㄏㄟ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="F204" s="15" t="str"/>
+    </x:row>
+    <x:row r="205" ht="15" hidden="0" customHeight="1">
+      <x:c r="A205" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B205" s="15" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C205" s="16" t="str">
+        <x:v>pink</x:v>
+      </x:c>
+      <x:c r="D205" s="16" t="str">
+        <x:v>粉紅色</x:v>
+      </x:c>
+      <x:c r="E205" s="16" t="str">
+        <x:v>ㄈㄣˇ ㄏㄨㄥˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="F205" s="15" t="str"/>
+    </x:row>
+    <x:row r="206" ht="15" hidden="0" customHeight="1">
+      <x:c r="A206" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B206" s="15" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C206" s="16" t="str">
+        <x:v>purple</x:v>
+      </x:c>
+      <x:c r="D206" s="16" t="str">
+        <x:v>紫色</x:v>
+      </x:c>
+      <x:c r="E206" s="16" t="str">
+        <x:v>ㄗˇ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="F206" s="15" t="str"/>
+    </x:row>
+    <x:row r="207" ht="15" hidden="0" customHeight="1">
+      <x:c r="A207" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B207" s="15" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C207" s="16" t="str">
+        <x:v>pretty</x:v>
+      </x:c>
+      <x:c r="D207" s="16" t="str">
+        <x:v>漂亮的</x:v>
+      </x:c>
+      <x:c r="E207" s="16" t="str">
+        <x:v>ㄆㄧㄠˋ ㄌㄧㄤˋ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="F207" s="15" t="str"/>
+    </x:row>
+    <x:row r="208" ht="15" hidden="0" customHeight="1">
+      <x:c r="A208" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B208" s="15" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C208" s="16" t="str">
+        <x:v>star</x:v>
+      </x:c>
+      <x:c r="D208" s="16" t="str">
+        <x:v>星星</x:v>
+      </x:c>
+      <x:c r="E208" s="16" t="str">
+        <x:v>ㄒㄧㄥ ㄒㄧㄥ</x:v>
+      </x:c>
+      <x:c r="F208" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="15" hidden="0" customHeight="1">
+      <x:c r="A209" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B209" s="15" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C209" s="16" t="str">
+        <x:v>triangle</x:v>
+      </x:c>
+      <x:c r="D209" s="16" t="str">
+        <x:v>三角形</x:v>
+      </x:c>
+      <x:c r="E209" s="16" t="str">
+        <x:v>ㄙㄢ ㄐㄧㄠˇ ㄒㄧㄥˊ</x:v>
+      </x:c>
+      <x:c r="F209" s="15" t="str"/>
+    </x:row>
+    <x:row r="210" ht="15" hidden="0" customHeight="1">
+      <x:c r="A210" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B210" s="15" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C210" s="16" t="str">
+        <x:v>little</x:v>
+      </x:c>
+      <x:c r="D210" s="16" t="str">
+        <x:v>小的</x:v>
+      </x:c>
+      <x:c r="E210" s="16" t="str">
+        <x:v>ㄒㄧㄠˇ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="F210" s="15" t="str"/>
+    </x:row>
+    <x:row r="211" ht="15" hidden="0" customHeight="1">
+      <x:c r="A211" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B211" s="15" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C211" s="16" t="str">
+        <x:v>or</x:v>
+      </x:c>
+      <x:c r="D211" s="16" t="str">
+        <x:v>或者</x:v>
+      </x:c>
+      <x:c r="E211" s="16" t="str">
+        <x:v>ㄏㄨㄛˋ ㄓㄜˇ</x:v>
+      </x:c>
+      <x:c r="F211" s="15" t="str"/>
+    </x:row>
+    <x:row r="212" ht="15" hidden="0" customHeight="1">
+      <x:c r="A212" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B212" s="15" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C212" s="16" t="str">
+        <x:v>shout</x:v>
+      </x:c>
+      <x:c r="D212" s="16" t="str">
+        <x:v>大喊</x:v>
+      </x:c>
+      <x:c r="E212" s="16" t="str">
+        <x:v>ㄉㄚˋ ㄏㄢˇ</x:v>
+      </x:c>
+      <x:c r="F212" s="15" t="str"/>
+    </x:row>
+    <x:row r="213" ht="15" hidden="0" customHeight="1">
+      <x:c r="A213" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B213" s="15" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C213" s="16" t="str">
+        <x:v>maybe</x:v>
+      </x:c>
+      <x:c r="D213" s="16" t="str">
+        <x:v>也許、可能</x:v>
+      </x:c>
+      <x:c r="E213" s="16" t="str">
+        <x:v>ㄧㄝˇ ㄒㄩˇ、ㄎㄜˇ ㄋㄥˊ</x:v>
+      </x:c>
+      <x:c r="F213" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="15" hidden="0" customHeight="1">
+      <x:c r="A214" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B214" s="15" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C214" s="16" t="str">
+        <x:v>dinosaur</x:v>
+      </x:c>
+      <x:c r="D214" s="16" t="str">
+        <x:v>恐龍</x:v>
+      </x:c>
+      <x:c r="E214" s="16" t="str">
+        <x:v>ㄎㄨㄥˇ ㄌㄨㄥˊ</x:v>
+      </x:c>
+      <x:c r="F214" s="15" t="str"/>
+    </x:row>
+    <x:row r="215" ht="15" hidden="0" customHeight="1">
+      <x:c r="A215" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B215" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C215" s="16" t="str">
+        <x:v>airplane</x:v>
+      </x:c>
+      <x:c r="D215" s="16" t="str">
+        <x:v>飛機</x:v>
+      </x:c>
+      <x:c r="E215" s="16" t="str">
+        <x:v>ㄈㄟ ㄐㄧ</x:v>
+      </x:c>
+      <x:c r="F215" s="15" t="str"/>
+    </x:row>
+    <x:row r="216" ht="15" hidden="0" customHeight="1">
+      <x:c r="A216" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B216" s="15" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C216" s="16" t="str">
+        <x:v>spot</x:v>
+      </x:c>
+      <x:c r="D216" s="16" t="str">
+        <x:v>斑點</x:v>
+      </x:c>
+      <x:c r="E216" s="16" t="str">
+        <x:v>ㄅㄢ ㄉㄧㄢˇ</x:v>
+      </x:c>
+      <x:c r="F216" s="15" t="str"/>
+    </x:row>
+    <x:row r="217" ht="15" hidden="0" customHeight="1">
+      <x:c r="A217" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B217" s="15" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C217" s="16" t="str">
+        <x:v>everywhere</x:v>
+      </x:c>
+      <x:c r="D217" s="16" t="str">
+        <x:v>到處</x:v>
+      </x:c>
+      <x:c r="E217" s="16" t="str">
+        <x:v>ㄉㄠˋ ㄔㄨˋ</x:v>
+      </x:c>
+      <x:c r="F217" s="15" t="str"/>
+    </x:row>
+    <x:row r="218" ht="15" hidden="0" customHeight="1">
+      <x:c r="A218" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B218" s="15" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C218" s="16" t="str">
+        <x:v>check</x:v>
+      </x:c>
+      <x:c r="D218" s="16" t="str">
+        <x:v>檢查</x:v>
+      </x:c>
+      <x:c r="E218" s="16" t="str">
+        <x:v>ㄐㄧㄢˇ ㄔㄚˊ</x:v>
+      </x:c>
+      <x:c r="F218" s="15" t="str"/>
+    </x:row>
+    <x:row r="219" ht="15" hidden="0" customHeight="1">
+      <x:c r="A219" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B219" s="15" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="C219" s="16" t="str">
+        <x:v>below</x:v>
+      </x:c>
+      <x:c r="D219" s="16" t="str">
+        <x:v>在下面</x:v>
+      </x:c>
+      <x:c r="E219" s="16" t="str">
+        <x:v>ㄗㄞˋ ㄒㄧㄚˋ ㄇㄧㄢˋ</x:v>
+      </x:c>
+      <x:c r="F219" s="15" t="str"/>
+    </x:row>
+    <x:row r="220" ht="15" hidden="0" customHeight="1">
+      <x:c r="A220" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B220" s="15" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C220" s="16" t="str">
+        <x:v>grass</x:v>
+      </x:c>
+      <x:c r="D220" s="16" t="str">
+        <x:v>草</x:v>
+      </x:c>
+      <x:c r="E220" s="16" t="str">
+        <x:v>ㄘㄠˇ</x:v>
+      </x:c>
+      <x:c r="F220" s="15" t="str"/>
+    </x:row>
+    <x:row r="221" ht="15" hidden="0" customHeight="1">
+      <x:c r="A221" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B221" s="15" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C221" s="16" t="str">
+        <x:v>butterfly</x:v>
+      </x:c>
+      <x:c r="D221" s="16" t="str">
+        <x:v>蝴蝶</x:v>
+      </x:c>
+      <x:c r="E221" s="16" t="str">
+        <x:v>ㄏㄨˊ ㄉㄧㄝˊ</x:v>
+      </x:c>
+      <x:c r="F221" s="15" t="str"/>
+    </x:row>
+    <x:row r="222" ht="15" hidden="0" customHeight="1">
+      <x:c r="A222" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B222" s="15" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C222" s="16" t="str">
+        <x:v>big / bigger</x:v>
+      </x:c>
+      <x:c r="D222" s="16" t="str">
+        <x:v>大的／更大的</x:v>
+      </x:c>
+      <x:c r="E222" s="16" t="str">
+        <x:v>ㄉㄚˋ ㄉㄜ˙／ㄍㄥˋ ㄉㄚˋ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="F222" s="15" t="str"/>
+    </x:row>
+    <x:row r="223" ht="15" hidden="0" customHeight="1">
+      <x:c r="A223" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B223" s="15" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C223" s="16" t="str">
+        <x:v>small</x:v>
+      </x:c>
+      <x:c r="D223" s="16" t="str">
+        <x:v>小的</x:v>
+      </x:c>
+      <x:c r="E223" s="16" t="str">
+        <x:v>ㄒㄧㄠˇ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="F223" s="15" t="str"/>
+    </x:row>
+    <x:row r="224" ht="15" hidden="0" customHeight="1">
+      <x:c r="A224" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B224" s="15" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="C224" s="16" t="str">
+        <x:v>more</x:v>
+      </x:c>
+      <x:c r="D224" s="16" t="str">
+        <x:v>更多</x:v>
+      </x:c>
+      <x:c r="E224" s="16" t="str">
+        <x:v>ㄍㄥˋ ㄉㄨㄛ</x:v>
+      </x:c>
+      <x:c r="F224" s="15" t="str">
+        <x:v>**</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="15" hidden="0" customHeight="1">
+      <x:c r="A225" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B225" s="15" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="C225" s="16" t="str">
+        <x:v>can</x:v>
+      </x:c>
+      <x:c r="D225" s="16" t="str">
+        <x:v>能、可以</x:v>
+      </x:c>
+      <x:c r="E225" s="16" t="str">
+        <x:v>ㄋㄥˊ、ㄎㄜˇ ㄧˇ</x:v>
+      </x:c>
+      <x:c r="F225" s="15" t="str"/>
+    </x:row>
+    <x:row r="226" ht="15" hidden="0" customHeight="1">
+      <x:c r="A226" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B226" s="15" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C226" s="16" t="str">
+        <x:v>paint</x:v>
+      </x:c>
+      <x:c r="D226" s="16" t="str">
+        <x:v>畫、塗顏料</x:v>
+      </x:c>
+      <x:c r="E226" s="16" t="str">
+        <x:v>ㄏㄨㄚˋ、ㄊㄨˊ ㄧㄢˊ ㄌㄧㄠˋ</x:v>
+      </x:c>
+      <x:c r="F226" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="15" hidden="0" customHeight="1">
+      <x:c r="A227" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B227" s="15" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C227" s="16" t="str">
+        <x:v>conclusion</x:v>
+      </x:c>
+      <x:c r="D227" s="16" t="str">
+        <x:v>結論</x:v>
+      </x:c>
+      <x:c r="E227" s="16" t="str">
+        <x:v>ㄐㄧㄝˊ ㄌㄨㄣˋ</x:v>
+      </x:c>
+      <x:c r="F227" s="15" t="str"/>
+    </x:row>
+    <x:row r="228" ht="15" hidden="0" customHeight="1">
+      <x:c r="A228" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B228" s="15" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C228" s="16" t="str">
+        <x:v>know</x:v>
+      </x:c>
+      <x:c r="D228" s="16" t="str">
+        <x:v>知道</x:v>
+      </x:c>
+      <x:c r="E228" s="16" t="str">
+        <x:v>ㄓ ㄉㄠˋ</x:v>
+      </x:c>
+      <x:c r="F228" s="15" t="str"/>
+    </x:row>
+    <x:row r="229" ht="15" hidden="0" customHeight="1">
+      <x:c r="A229" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B229" s="15" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C229" s="16" t="str">
+        <x:v>wheel</x:v>
+      </x:c>
+      <x:c r="D229" s="16" t="str">
+        <x:v>輪子</x:v>
+      </x:c>
+      <x:c r="E229" s="16" t="str">
+        <x:v>ㄌㄨㄣˊ ㄗ˙</x:v>
+      </x:c>
+      <x:c r="F229" s="15" t="str"/>
+    </x:row>
+    <x:row r="230" ht="15" hidden="0" customHeight="1">
+      <x:c r="A230" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B230" s="15" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C230" s="16" t="str">
+        <x:v>between</x:v>
+      </x:c>
+      <x:c r="D230" s="16" t="str">
+        <x:v>在……之間</x:v>
+      </x:c>
+      <x:c r="E230" s="16" t="str">
+        <x:v>ㄗㄞˋ……ㄓ ㄐㄧㄢ</x:v>
+      </x:c>
+      <x:c r="F230" s="15" t="str"/>
+    </x:row>
+    <x:row r="231" ht="15" hidden="0" customHeight="1">
+      <x:c r="A231" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B231" s="15" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C231" s="16" t="str">
+        <x:v>like</x:v>
+      </x:c>
+      <x:c r="D231" s="16" t="str">
+        <x:v>喜歡、像</x:v>
+      </x:c>
+      <x:c r="E231" s="16" t="str">
+        <x:v>ㄒㄧˇ ㄏㄨㄢ、ㄒㄧㄤˋ</x:v>
+      </x:c>
+      <x:c r="F231" s="15" t="str"/>
+    </x:row>
+    <x:row r="232" ht="15" hidden="0" customHeight="1">
+      <x:c r="A232" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B232" s="15" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C232" s="16" t="str">
+        <x:v>close</x:v>
+      </x:c>
+      <x:c r="D232" s="16" t="str">
+        <x:v>關上、靠近</x:v>
+      </x:c>
+      <x:c r="E232" s="16" t="str">
+        <x:v>ㄍㄨㄢ ㄕㄤˋ、ㄎㄠˋ ㄐㄧㄣˋ</x:v>
+      </x:c>
+      <x:c r="F232" s="15" t="str"/>
+    </x:row>
+    <x:row r="233" ht="15" hidden="0" customHeight="1">
+      <x:c r="A233" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B233" s="15" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="C233" s="16" t="str">
+        <x:v>figure out</x:v>
+      </x:c>
+      <x:c r="D233" s="16" t="str">
+        <x:v>想出、弄清楚</x:v>
+      </x:c>
+      <x:c r="E233" s="16" t="str">
+        <x:v>ㄒㄧㄤˇ ㄔㄨ、ㄋㄨㄥˋ ㄑㄧㄥ ㄔㄨˇ</x:v>
+      </x:c>
+      <x:c r="F233" s="15" t="str"/>
+    </x:row>
+    <x:row r="234" ht="15" hidden="0" customHeight="1">
+      <x:c r="A234" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B234" s="15" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="C234" s="16" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="D234" s="16" t="str">
+        <x:v>數數</x:v>
+      </x:c>
+      <x:c r="E234" s="16" t="str">
+        <x:v>ㄕㄨˇ ㄕㄨˋ</x:v>
+      </x:c>
+      <x:c r="F234" s="15" t="str"/>
+    </x:row>
+    <x:row r="235" ht="15" hidden="0" customHeight="1">
+      <x:c r="A235" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B235" s="15" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="C235" s="16" t="str">
+        <x:v>far</x:v>
+      </x:c>
+      <x:c r="D235" s="16" t="str">
+        <x:v>遠的</x:v>
+      </x:c>
+      <x:c r="E235" s="16" t="str">
+        <x:v>ㄩㄢˇ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="F235" s="15" t="str"/>
+    </x:row>
+    <x:row r="236" ht="15" hidden="0" customHeight="1">
+      <x:c r="A236" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B236" s="15" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C236" s="16" t="str">
+        <x:v>away from</x:v>
+      </x:c>
+      <x:c r="D236" s="16" t="str">
+        <x:v>遠離</x:v>
+      </x:c>
+      <x:c r="E236" s="16" t="str">
+        <x:v>ㄩㄢˇ ㄌㄧˊ</x:v>
+      </x:c>
+      <x:c r="F236" s="15" t="str"/>
+    </x:row>
+    <x:row r="237" ht="15" hidden="0" customHeight="1">
+      <x:c r="A237" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B237" s="15" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="C237" s="16" t="str">
+        <x:v>gorilla</x:v>
+      </x:c>
+      <x:c r="D237" s="16" t="str">
+        <x:v>大猩猩</x:v>
+      </x:c>
+      <x:c r="E237" s="16" t="str">
+        <x:v>ㄉㄚˋ ㄒㄧㄥ ㄒㄧㄥ</x:v>
+      </x:c>
+      <x:c r="F237" s="15" t="str"/>
+    </x:row>
+    <x:row r="238" ht="15" hidden="0" customHeight="1">
+      <x:c r="A238" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B238" s="15" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C238" s="16" t="str">
+        <x:v>iguana</x:v>
+      </x:c>
+      <x:c r="D238" s="16" t="str">
+        <x:v>鬣蜥</x:v>
+      </x:c>
+      <x:c r="E238" s="16" t="str">
+        <x:v>ㄌㄧㄝˋ ㄒㄧ</x:v>
+      </x:c>
+      <x:c r="F238" s="15" t="str"/>
+    </x:row>
+    <x:row r="239" ht="15" hidden="0" customHeight="1">
+      <x:c r="A239" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B239" s="15" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="C239" s="16" t="str">
+        <x:v>horse</x:v>
+      </x:c>
+      <x:c r="D239" s="16" t="str">
+        <x:v>馬</x:v>
+      </x:c>
+      <x:c r="E239" s="16" t="str">
+        <x:v>ㄇㄚˇ</x:v>
+      </x:c>
+      <x:c r="F239" s="15" t="str"/>
+    </x:row>
+    <x:row r="240" ht="15" hidden="0" customHeight="1">
+      <x:c r="A240" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B240" s="15" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="C240" s="16" t="str">
+        <x:v>house</x:v>
+      </x:c>
+      <x:c r="D240" s="16" t="str">
+        <x:v>房子、家</x:v>
+      </x:c>
+      <x:c r="E240" s="16" t="str">
+        <x:v>ㄈㄤˊ ㄗ˙、ㄐㄧㄚ</x:v>
+      </x:c>
+      <x:c r="F240" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="15" hidden="0" customHeight="1">
+      <x:c r="A241" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B241" s="15" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C241" s="16" t="str">
+        <x:v>run</x:v>
+      </x:c>
+      <x:c r="D241" s="16" t="str">
+        <x:v>跑</x:v>
+      </x:c>
+      <x:c r="E241" s="16" t="str">
+        <x:v>ㄆㄠˇ</x:v>
+      </x:c>
+      <x:c r="F241" s="15" t="str"/>
+    </x:row>
+    <x:row r="242" ht="15" hidden="0" customHeight="1">
+      <x:c r="A242" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B242" s="15" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="C242" s="16" t="str">
+        <x:v>pound</x:v>
+      </x:c>
+      <x:c r="D242" s="16" t="str">
+        <x:v>磅、重擊</x:v>
+      </x:c>
+      <x:c r="E242" s="16" t="str">
+        <x:v>ㄅㄤˋ、ㄓㄨㄥˋ ㄐㄧˊ</x:v>
+      </x:c>
+      <x:c r="F242" s="15" t="str"/>
+    </x:row>
+    <x:row r="243" ht="15" hidden="0" customHeight="1">
+      <x:c r="A243" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B243" s="15" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="C243" s="16" t="str">
+        <x:v>lick</x:v>
+      </x:c>
+      <x:c r="D243" s="16" t="str">
+        <x:v>舔</x:v>
+      </x:c>
+      <x:c r="E243" s="16" t="str">
+        <x:v>ㄊㄧㄢˇ</x:v>
+      </x:c>
+      <x:c r="F243" s="15" t="str"/>
+    </x:row>
+    <x:row r="244" ht="15" hidden="0" customHeight="1">
+      <x:c r="A244" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B244" s="15" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="C244" s="16" t="str">
+        <x:v>grrr</x:v>
+      </x:c>
+      <x:c r="D244" s="16" t="str">
+        <x:v>吼！</x:v>
+      </x:c>
+      <x:c r="E244" s="16" t="str">
+        <x:v>ㄏㄡˇ</x:v>
+      </x:c>
+      <x:c r="F244" s="15" t="str"/>
+    </x:row>
+    <x:row r="245" ht="15" hidden="0" customHeight="1">
+      <x:c r="A245" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B245" s="15" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C245" s="16" t="str">
+        <x:v>goat</x:v>
+      </x:c>
+      <x:c r="D245" s="16" t="str">
+        <x:v>山羊</x:v>
+      </x:c>
+      <x:c r="E245" s="16" t="str">
+        <x:v>ㄕㄢ ㄧㄤˊ</x:v>
+      </x:c>
+      <x:c r="F245" s="15" t="str"/>
+    </x:row>
+    <x:row r="246" ht="15" hidden="0" customHeight="1">
+      <x:c r="A246" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B246" s="15" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C246" s="16" t="str">
+        <x:v>guitar</x:v>
+      </x:c>
+      <x:c r="D246" s="16" t="str">
+        <x:v>吉他</x:v>
+      </x:c>
+      <x:c r="E246" s="16" t="str">
+        <x:v>ㄐㄧˊ ㄊㄚ</x:v>
+      </x:c>
+      <x:c r="F246" s="15" t="str"/>
+    </x:row>
+    <x:row r="247" ht="15" hidden="0" customHeight="1">
+      <x:c r="A247" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B247" s="15" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C247" s="16" t="str">
+        <x:v>hat</x:v>
+      </x:c>
+      <x:c r="D247" s="16" t="str">
+        <x:v>帽子</x:v>
+      </x:c>
+      <x:c r="E247" s="16" t="str">
+        <x:v>ㄇㄠˋ ㄗ˙</x:v>
+      </x:c>
+      <x:c r="F247" s="15" t="str"/>
+    </x:row>
+    <x:row r="248" ht="15" hidden="0" customHeight="1">
+      <x:c r="A248" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B248" s="15" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="C248" s="16" t="str">
+        <x:v>ink</x:v>
+      </x:c>
+      <x:c r="D248" s="16" t="str">
+        <x:v>墨水</x:v>
+      </x:c>
+      <x:c r="E248" s="16" t="str">
+        <x:v>ㄇㄛˋ ㄕㄨㄟˇ</x:v>
+      </x:c>
+      <x:c r="F248" s="15" t="str"/>
+    </x:row>
+    <x:row r="249" ht="15" hidden="0" customHeight="1">
+      <x:c r="A249" s="15" t="str">
+        <x:v>Lesson 4</x:v>
+      </x:c>
+      <x:c r="B249" s="15" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="C249" s="16" t="str">
+        <x:v>igloo</x:v>
+      </x:c>
+      <x:c r="D249" s="16" t="str">
+        <x:v>冰屋</x:v>
+      </x:c>
+      <x:c r="E249" s="16" t="str">
+        <x:v>ㄅㄧㄥ ㄨ</x:v>
+      </x:c>
+      <x:c r="F249" s="15" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:F2"/>
     <x:mergeCell ref="A3:F3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="F5:F191">
+  <x:conditionalFormatting sqref="F5:F249">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="*"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R373949e56561446a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23d21098bb854c95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5132,7 +6220,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8048cbb821764427"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b7be52edd6c4fba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6318,7 +7406,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f178449749d4ab9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1569580fb3e54500"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6967,7 +8055,950 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5e7c5a26bac4cd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd7199024af04e29"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFA64D79"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Lesson 4 英文單字表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="4" t="str">
+        <x:v>重複標記：* 代表第二次出現；** 代表第三次出現。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="13" t="str">
+        <x:v>編號</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="str">
+        <x:v>英文</x:v>
+      </x:c>
+      <x:c r="C4" s="13" t="str">
+        <x:v>繁體中文</x:v>
+      </x:c>
+      <x:c r="D4" s="13" t="str">
+        <x:v>注音</x:v>
+      </x:c>
+      <x:c r="E4" s="13" t="str">
+        <x:v>重複標記</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="16" t="str">
+        <x:v>take a look</x:v>
+      </x:c>
+      <x:c r="C5" s="16" t="str">
+        <x:v>看一看</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="str">
+        <x:v>ㄎㄢˋ ㄧˊ ㄎㄢˋ</x:v>
+      </x:c>
+      <x:c r="E5" s="15" t="str"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="str">
+        <x:v>shirt</x:v>
+      </x:c>
+      <x:c r="C6" s="16" t="str">
+        <x:v>襯衫</x:v>
+      </x:c>
+      <x:c r="D6" s="16" t="str">
+        <x:v>ㄔㄣˋ ㄕㄢ</x:v>
+      </x:c>
+      <x:c r="E6" s="15" t="str"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>shelf</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="str">
+        <x:v>架子</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>ㄐㄧㄚˋ ㄗ˙</x:v>
+      </x:c>
+      <x:c r="E7" s="15" t="str"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>flower</x:v>
+      </x:c>
+      <x:c r="C8" s="16" t="str">
+        <x:v>花</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="str">
+        <x:v>ㄏㄨㄚ</x:v>
+      </x:c>
+      <x:c r="E8" s="15" t="str"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="str">
+        <x:v>wear / wearing</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="str">
+        <x:v>穿／正在穿</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>ㄔㄨㄢ／ㄓㄥˋ ㄗㄞˋ ㄔㄨㄢ</x:v>
+      </x:c>
+      <x:c r="E9" s="15" t="str"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="str">
+        <x:v>jacket</x:v>
+      </x:c>
+      <x:c r="C10" s="16" t="str">
+        <x:v>夾克、外套</x:v>
+      </x:c>
+      <x:c r="D10" s="16" t="str">
+        <x:v>ㄐㄧㄚˊ ㄎㄜˋ、ㄨㄞˋ ㄊㄠˋ</x:v>
+      </x:c>
+      <x:c r="E10" s="15" t="str"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="15" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>red</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>紅色</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="str">
+        <x:v>ㄏㄨㄥˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="E11" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="str">
+        <x:v>yellow</x:v>
+      </x:c>
+      <x:c r="C12" s="16" t="str">
+        <x:v>黃色</x:v>
+      </x:c>
+      <x:c r="D12" s="16" t="str">
+        <x:v>ㄏㄨㄤˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="E12" s="15" t="str"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="15" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="str">
+        <x:v>blue</x:v>
+      </x:c>
+      <x:c r="C13" s="16" t="str">
+        <x:v>藍色</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="str">
+        <x:v>ㄌㄢˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="E13" s="15" t="str"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="15" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="str">
+        <x:v>green</x:v>
+      </x:c>
+      <x:c r="C14" s="16" t="str">
+        <x:v>綠色</x:v>
+      </x:c>
+      <x:c r="D14" s="16" t="str">
+        <x:v>ㄌㄩˋ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="E14" s="15" t="str"/>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="15" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="str">
+        <x:v>orange</x:v>
+      </x:c>
+      <x:c r="C15" s="16" t="str">
+        <x:v>橘色</x:v>
+      </x:c>
+      <x:c r="D15" s="16" t="str">
+        <x:v>ㄐㄩˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="E15" s="15" t="str"/>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B16" s="16" t="str">
+        <x:v>white</x:v>
+      </x:c>
+      <x:c r="C16" s="16" t="str">
+        <x:v>白色</x:v>
+      </x:c>
+      <x:c r="D16" s="16" t="str">
+        <x:v>ㄅㄞˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="E16" s="15" t="str"/>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="15" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B17" s="16" t="str">
+        <x:v>black</x:v>
+      </x:c>
+      <x:c r="C17" s="16" t="str">
+        <x:v>黑色</x:v>
+      </x:c>
+      <x:c r="D17" s="16" t="str">
+        <x:v>ㄏㄟ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="E17" s="15" t="str"/>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="15" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B18" s="16" t="str">
+        <x:v>pink</x:v>
+      </x:c>
+      <x:c r="C18" s="16" t="str">
+        <x:v>粉紅色</x:v>
+      </x:c>
+      <x:c r="D18" s="16" t="str">
+        <x:v>ㄈㄣˇ ㄏㄨㄥˊ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="E18" s="15" t="str"/>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="15" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B19" s="16" t="str">
+        <x:v>purple</x:v>
+      </x:c>
+      <x:c r="C19" s="16" t="str">
+        <x:v>紫色</x:v>
+      </x:c>
+      <x:c r="D19" s="16" t="str">
+        <x:v>ㄗˇ ㄙㄜˋ</x:v>
+      </x:c>
+      <x:c r="E19" s="15" t="str"/>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="15" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B20" s="16" t="str">
+        <x:v>pretty</x:v>
+      </x:c>
+      <x:c r="C20" s="16" t="str">
+        <x:v>漂亮的</x:v>
+      </x:c>
+      <x:c r="D20" s="16" t="str">
+        <x:v>ㄆㄧㄠˋ ㄌㄧㄤˋ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="E20" s="15" t="str"/>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="15" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B21" s="16" t="str">
+        <x:v>star</x:v>
+      </x:c>
+      <x:c r="C21" s="16" t="str">
+        <x:v>星星</x:v>
+      </x:c>
+      <x:c r="D21" s="16" t="str">
+        <x:v>ㄒㄧㄥ ㄒㄧㄥ</x:v>
+      </x:c>
+      <x:c r="E21" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="15" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B22" s="16" t="str">
+        <x:v>triangle</x:v>
+      </x:c>
+      <x:c r="C22" s="16" t="str">
+        <x:v>三角形</x:v>
+      </x:c>
+      <x:c r="D22" s="16" t="str">
+        <x:v>ㄙㄢ ㄐㄧㄠˇ ㄒㄧㄥˊ</x:v>
+      </x:c>
+      <x:c r="E22" s="15" t="str"/>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="15" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="str">
+        <x:v>little</x:v>
+      </x:c>
+      <x:c r="C23" s="16" t="str">
+        <x:v>小的</x:v>
+      </x:c>
+      <x:c r="D23" s="16" t="str">
+        <x:v>ㄒㄧㄠˇ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="E23" s="15" t="str"/>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="15" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B24" s="16" t="str">
+        <x:v>or</x:v>
+      </x:c>
+      <x:c r="C24" s="16" t="str">
+        <x:v>或者</x:v>
+      </x:c>
+      <x:c r="D24" s="16" t="str">
+        <x:v>ㄏㄨㄛˋ ㄓㄜˇ</x:v>
+      </x:c>
+      <x:c r="E24" s="15" t="str"/>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="15" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B25" s="16" t="str">
+        <x:v>shout</x:v>
+      </x:c>
+      <x:c r="C25" s="16" t="str">
+        <x:v>大喊</x:v>
+      </x:c>
+      <x:c r="D25" s="16" t="str">
+        <x:v>ㄉㄚˋ ㄏㄢˇ</x:v>
+      </x:c>
+      <x:c r="E25" s="15" t="str"/>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="15" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B26" s="16" t="str">
+        <x:v>maybe</x:v>
+      </x:c>
+      <x:c r="C26" s="16" t="str">
+        <x:v>也許、可能</x:v>
+      </x:c>
+      <x:c r="D26" s="16" t="str">
+        <x:v>ㄧㄝˇ ㄒㄩˇ、ㄎㄜˇ ㄋㄥˊ</x:v>
+      </x:c>
+      <x:c r="E26" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="15" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B27" s="16" t="str">
+        <x:v>dinosaur</x:v>
+      </x:c>
+      <x:c r="C27" s="16" t="str">
+        <x:v>恐龍</x:v>
+      </x:c>
+      <x:c r="D27" s="16" t="str">
+        <x:v>ㄎㄨㄥˇ ㄌㄨㄥˊ</x:v>
+      </x:c>
+      <x:c r="E27" s="15" t="str"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B28" s="16" t="str">
+        <x:v>airplane</x:v>
+      </x:c>
+      <x:c r="C28" s="16" t="str">
+        <x:v>飛機</x:v>
+      </x:c>
+      <x:c r="D28" s="16" t="str">
+        <x:v>ㄈㄟ ㄐㄧ</x:v>
+      </x:c>
+      <x:c r="E28" s="15" t="str"/>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="15" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B29" s="16" t="str">
+        <x:v>spot</x:v>
+      </x:c>
+      <x:c r="C29" s="16" t="str">
+        <x:v>斑點</x:v>
+      </x:c>
+      <x:c r="D29" s="16" t="str">
+        <x:v>ㄅㄢ ㄉㄧㄢˇ</x:v>
+      </x:c>
+      <x:c r="E29" s="15" t="str"/>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="15" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B30" s="16" t="str">
+        <x:v>everywhere</x:v>
+      </x:c>
+      <x:c r="C30" s="16" t="str">
+        <x:v>到處</x:v>
+      </x:c>
+      <x:c r="D30" s="16" t="str">
+        <x:v>ㄉㄠˋ ㄔㄨˋ</x:v>
+      </x:c>
+      <x:c r="E30" s="15" t="str"/>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="15" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B31" s="16" t="str">
+        <x:v>check</x:v>
+      </x:c>
+      <x:c r="C31" s="16" t="str">
+        <x:v>檢查</x:v>
+      </x:c>
+      <x:c r="D31" s="16" t="str">
+        <x:v>ㄐㄧㄢˇ ㄔㄚˊ</x:v>
+      </x:c>
+      <x:c r="E31" s="15" t="str"/>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="15" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B32" s="16" t="str">
+        <x:v>below</x:v>
+      </x:c>
+      <x:c r="C32" s="16" t="str">
+        <x:v>在下面</x:v>
+      </x:c>
+      <x:c r="D32" s="16" t="str">
+        <x:v>ㄗㄞˋ ㄒㄧㄚˋ ㄇㄧㄢˋ</x:v>
+      </x:c>
+      <x:c r="E32" s="15" t="str"/>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="15" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B33" s="16" t="str">
+        <x:v>grass</x:v>
+      </x:c>
+      <x:c r="C33" s="16" t="str">
+        <x:v>草</x:v>
+      </x:c>
+      <x:c r="D33" s="16" t="str">
+        <x:v>ㄘㄠˇ</x:v>
+      </x:c>
+      <x:c r="E33" s="15" t="str"/>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="15" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B34" s="16" t="str">
+        <x:v>butterfly</x:v>
+      </x:c>
+      <x:c r="C34" s="16" t="str">
+        <x:v>蝴蝶</x:v>
+      </x:c>
+      <x:c r="D34" s="16" t="str">
+        <x:v>ㄏㄨˊ ㄉㄧㄝˊ</x:v>
+      </x:c>
+      <x:c r="E34" s="15" t="str"/>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="A35" s="15" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B35" s="16" t="str">
+        <x:v>big / bigger</x:v>
+      </x:c>
+      <x:c r="C35" s="16" t="str">
+        <x:v>大的／更大的</x:v>
+      </x:c>
+      <x:c r="D35" s="16" t="str">
+        <x:v>ㄉㄚˋ ㄉㄜ˙／ㄍㄥˋ ㄉㄚˋ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="E35" s="15" t="str"/>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="15" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B36" s="16" t="str">
+        <x:v>small</x:v>
+      </x:c>
+      <x:c r="C36" s="16" t="str">
+        <x:v>小的</x:v>
+      </x:c>
+      <x:c r="D36" s="16" t="str">
+        <x:v>ㄒㄧㄠˇ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="E36" s="15" t="str"/>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="15" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B37" s="16" t="str">
+        <x:v>more</x:v>
+      </x:c>
+      <x:c r="C37" s="16" t="str">
+        <x:v>更多</x:v>
+      </x:c>
+      <x:c r="D37" s="16" t="str">
+        <x:v>ㄍㄥˋ ㄉㄨㄛ</x:v>
+      </x:c>
+      <x:c r="E37" s="15" t="str">
+        <x:v>**</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="15" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B38" s="16" t="str">
+        <x:v>can</x:v>
+      </x:c>
+      <x:c r="C38" s="16" t="str">
+        <x:v>能、可以</x:v>
+      </x:c>
+      <x:c r="D38" s="16" t="str">
+        <x:v>ㄋㄥˊ、ㄎㄜˇ ㄧˇ</x:v>
+      </x:c>
+      <x:c r="E38" s="15" t="str"/>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="15" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B39" s="16" t="str">
+        <x:v>paint</x:v>
+      </x:c>
+      <x:c r="C39" s="16" t="str">
+        <x:v>畫、塗顏料</x:v>
+      </x:c>
+      <x:c r="D39" s="16" t="str">
+        <x:v>ㄏㄨㄚˋ、ㄊㄨˊ ㄧㄢˊ ㄌㄧㄠˋ</x:v>
+      </x:c>
+      <x:c r="E39" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="15" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B40" s="16" t="str">
+        <x:v>conclusion</x:v>
+      </x:c>
+      <x:c r="C40" s="16" t="str">
+        <x:v>結論</x:v>
+      </x:c>
+      <x:c r="D40" s="16" t="str">
+        <x:v>ㄐㄧㄝˊ ㄌㄨㄣˋ</x:v>
+      </x:c>
+      <x:c r="E40" s="15" t="str"/>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="A41" s="15" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B41" s="16" t="str">
+        <x:v>know</x:v>
+      </x:c>
+      <x:c r="C41" s="16" t="str">
+        <x:v>知道</x:v>
+      </x:c>
+      <x:c r="D41" s="16" t="str">
+        <x:v>ㄓ ㄉㄠˋ</x:v>
+      </x:c>
+      <x:c r="E41" s="15" t="str"/>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="15" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B42" s="16" t="str">
+        <x:v>wheel</x:v>
+      </x:c>
+      <x:c r="C42" s="16" t="str">
+        <x:v>輪子</x:v>
+      </x:c>
+      <x:c r="D42" s="16" t="str">
+        <x:v>ㄌㄨㄣˊ ㄗ˙</x:v>
+      </x:c>
+      <x:c r="E42" s="15" t="str"/>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="15" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B43" s="16" t="str">
+        <x:v>between</x:v>
+      </x:c>
+      <x:c r="C43" s="16" t="str">
+        <x:v>在……之間</x:v>
+      </x:c>
+      <x:c r="D43" s="16" t="str">
+        <x:v>ㄗㄞˋ……ㄓ ㄐㄧㄢ</x:v>
+      </x:c>
+      <x:c r="E43" s="15" t="str"/>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="15" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B44" s="16" t="str">
+        <x:v>like</x:v>
+      </x:c>
+      <x:c r="C44" s="16" t="str">
+        <x:v>喜歡、像</x:v>
+      </x:c>
+      <x:c r="D44" s="16" t="str">
+        <x:v>ㄒㄧˇ ㄏㄨㄢ、ㄒㄧㄤˋ</x:v>
+      </x:c>
+      <x:c r="E44" s="15" t="str"/>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="15" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B45" s="16" t="str">
+        <x:v>close</x:v>
+      </x:c>
+      <x:c r="C45" s="16" t="str">
+        <x:v>關上、靠近</x:v>
+      </x:c>
+      <x:c r="D45" s="16" t="str">
+        <x:v>ㄍㄨㄢ ㄕㄤˋ、ㄎㄠˋ ㄐㄧㄣˋ</x:v>
+      </x:c>
+      <x:c r="E45" s="15" t="str"/>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="15" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B46" s="16" t="str">
+        <x:v>figure out</x:v>
+      </x:c>
+      <x:c r="C46" s="16" t="str">
+        <x:v>想出、弄清楚</x:v>
+      </x:c>
+      <x:c r="D46" s="16" t="str">
+        <x:v>ㄒㄧㄤˇ ㄔㄨ、ㄋㄨㄥˋ ㄑㄧㄥ ㄔㄨˇ</x:v>
+      </x:c>
+      <x:c r="E46" s="15" t="str"/>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="15" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B47" s="16" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="C47" s="16" t="str">
+        <x:v>數數</x:v>
+      </x:c>
+      <x:c r="D47" s="16" t="str">
+        <x:v>ㄕㄨˇ ㄕㄨˋ</x:v>
+      </x:c>
+      <x:c r="E47" s="15" t="str"/>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="15" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="str">
+        <x:v>far</x:v>
+      </x:c>
+      <x:c r="C48" s="16" t="str">
+        <x:v>遠的</x:v>
+      </x:c>
+      <x:c r="D48" s="16" t="str">
+        <x:v>ㄩㄢˇ ㄉㄜ˙</x:v>
+      </x:c>
+      <x:c r="E48" s="15" t="str"/>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="15" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B49" s="16" t="str">
+        <x:v>away from</x:v>
+      </x:c>
+      <x:c r="C49" s="16" t="str">
+        <x:v>遠離</x:v>
+      </x:c>
+      <x:c r="D49" s="16" t="str">
+        <x:v>ㄩㄢˇ ㄌㄧˊ</x:v>
+      </x:c>
+      <x:c r="E49" s="15" t="str"/>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="15" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B50" s="16" t="str">
+        <x:v>gorilla</x:v>
+      </x:c>
+      <x:c r="C50" s="16" t="str">
+        <x:v>大猩猩</x:v>
+      </x:c>
+      <x:c r="D50" s="16" t="str">
+        <x:v>ㄉㄚˋ ㄒㄧㄥ ㄒㄧㄥ</x:v>
+      </x:c>
+      <x:c r="E50" s="15" t="str"/>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="15" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B51" s="16" t="str">
+        <x:v>iguana</x:v>
+      </x:c>
+      <x:c r="C51" s="16" t="str">
+        <x:v>鬣蜥</x:v>
+      </x:c>
+      <x:c r="D51" s="16" t="str">
+        <x:v>ㄌㄧㄝˋ ㄒㄧ</x:v>
+      </x:c>
+      <x:c r="E51" s="15" t="str"/>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="15" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B52" s="16" t="str">
+        <x:v>horse</x:v>
+      </x:c>
+      <x:c r="C52" s="16" t="str">
+        <x:v>馬</x:v>
+      </x:c>
+      <x:c r="D52" s="16" t="str">
+        <x:v>ㄇㄚˇ</x:v>
+      </x:c>
+      <x:c r="E52" s="15" t="str"/>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="15" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B53" s="16" t="str">
+        <x:v>house</x:v>
+      </x:c>
+      <x:c r="C53" s="16" t="str">
+        <x:v>房子、家</x:v>
+      </x:c>
+      <x:c r="D53" s="16" t="str">
+        <x:v>ㄈㄤˊ ㄗ˙、ㄐㄧㄚ</x:v>
+      </x:c>
+      <x:c r="E53" s="15" t="str">
+        <x:v>*</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="15" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B54" s="16" t="str">
+        <x:v>run</x:v>
+      </x:c>
+      <x:c r="C54" s="16" t="str">
+        <x:v>跑</x:v>
+      </x:c>
+      <x:c r="D54" s="16" t="str">
+        <x:v>ㄆㄠˇ</x:v>
+      </x:c>
+      <x:c r="E54" s="15" t="str"/>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="15" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B55" s="16" t="str">
+        <x:v>pound</x:v>
+      </x:c>
+      <x:c r="C55" s="16" t="str">
+        <x:v>磅、重擊</x:v>
+      </x:c>
+      <x:c r="D55" s="16" t="str">
+        <x:v>ㄅㄤˋ、ㄓㄨㄥˋ ㄐㄧˊ</x:v>
+      </x:c>
+      <x:c r="E55" s="15" t="str"/>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="15" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B56" s="16" t="str">
+        <x:v>lick</x:v>
+      </x:c>
+      <x:c r="C56" s="16" t="str">
+        <x:v>舔</x:v>
+      </x:c>
+      <x:c r="D56" s="16" t="str">
+        <x:v>ㄊㄧㄢˇ</x:v>
+      </x:c>
+      <x:c r="E56" s="15" t="str"/>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="15" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B57" s="16" t="str">
+        <x:v>grrr</x:v>
+      </x:c>
+      <x:c r="C57" s="16" t="str">
+        <x:v>吼！</x:v>
+      </x:c>
+      <x:c r="D57" s="16" t="str">
+        <x:v>ㄏㄡˇ</x:v>
+      </x:c>
+      <x:c r="E57" s="15" t="str"/>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="15" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B58" s="16" t="str">
+        <x:v>goat</x:v>
+      </x:c>
+      <x:c r="C58" s="16" t="str">
+        <x:v>山羊</x:v>
+      </x:c>
+      <x:c r="D58" s="16" t="str">
+        <x:v>ㄕㄢ ㄧㄤˊ</x:v>
+      </x:c>
+      <x:c r="E58" s="15" t="str"/>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="A59" s="15" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B59" s="16" t="str">
+        <x:v>guitar</x:v>
+      </x:c>
+      <x:c r="C59" s="16" t="str">
+        <x:v>吉他</x:v>
+      </x:c>
+      <x:c r="D59" s="16" t="str">
+        <x:v>ㄐㄧˊ ㄊㄚ</x:v>
+      </x:c>
+      <x:c r="E59" s="15" t="str"/>
+    </x:row>
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="A60" s="15" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B60" s="16" t="str">
+        <x:v>hat</x:v>
+      </x:c>
+      <x:c r="C60" s="16" t="str">
+        <x:v>帽子</x:v>
+      </x:c>
+      <x:c r="D60" s="16" t="str">
+        <x:v>ㄇㄠˋ ㄗ˙</x:v>
+      </x:c>
+      <x:c r="E60" s="15" t="str"/>
+    </x:row>
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
+      <x:c r="A61" s="15" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B61" s="16" t="str">
+        <x:v>ink</x:v>
+      </x:c>
+      <x:c r="C61" s="16" t="str">
+        <x:v>墨水</x:v>
+      </x:c>
+      <x:c r="D61" s="16" t="str">
+        <x:v>ㄇㄛˋ ㄕㄨㄟˇ</x:v>
+      </x:c>
+      <x:c r="E61" s="15" t="str"/>
+    </x:row>
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="A62" s="15" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B62" s="16" t="str">
+        <x:v>igloo</x:v>
+      </x:c>
+      <x:c r="C62" s="16" t="str">
+        <x:v>冰屋</x:v>
+      </x:c>
+      <x:c r="D62" s="16" t="str">
+        <x:v>ㄅㄧㄥ ㄨ</x:v>
+      </x:c>
+      <x:c r="E62" s="15" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A3:E3"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="A5:E62">
+    <x:cfRule type="expression" dxfId="7" priority="1">
+      <x:formula>MOD(ROW(),2)=1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E5:E62">
+    <x:cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="*"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f1285cc0e294708"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>